<commit_message>
chore(model): promote retrained model — AUC 0.7720 overall, May-only clean slice
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-23.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-23.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2411</v>
+        <v>2424</v>
       </c>
       <c r="E2" t="n">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="F2" t="n">
-        <v>2001</v>
+        <v>2008</v>
       </c>
       <c r="G2" t="n">
-        <v>17</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="E3" t="n">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="F3" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G3" t="n">
-        <v>66.09999999999999</v>
+        <v>67.09999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F4" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G4" t="n">
-        <v>31.7</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E5" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G5" t="n">
-        <v>57.7</v>
+        <v>59.4</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="E6" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F6" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="G6" t="n">
-        <v>47.5</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F7" t="n">
         <v>6</v>
       </c>
       <c r="G7" t="n">
-        <v>62.5</v>
+        <v>64.7</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>567</v>
+        <v>596</v>
       </c>
       <c r="E8" t="n">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="F8" t="n">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="G8" t="n">
-        <v>40.2</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>205</v>
+        <v>223</v>
       </c>
       <c r="E9" t="n">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="F9" t="n">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G9" t="n">
-        <v>61</v>
+        <v>60.1</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>496</v>
+        <v>573</v>
       </c>
       <c r="E10" t="n">
-        <v>315</v>
+        <v>350</v>
       </c>
       <c r="F10" t="n">
-        <v>181</v>
+        <v>223</v>
       </c>
       <c r="G10" t="n">
-        <v>63.5</v>
+        <v>61.1</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>286</v>
+        <v>336</v>
       </c>
       <c r="E11" t="n">
-        <v>181</v>
+        <v>215</v>
       </c>
       <c r="F11" t="n">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="G11" t="n">
-        <v>63.3</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12">
@@ -761,13 +761,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="E12" t="n">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="F12" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="G12" t="n">
         <v>61.4</v>
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="E13" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F13" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G13" t="n">
-        <v>60.9</v>
+        <v>61.5</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>162</v>
+        <v>206</v>
       </c>
       <c r="E14" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F14" t="n">
-        <v>122</v>
+        <v>160</v>
       </c>
       <c r="G14" t="n">
-        <v>24.7</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
+        <v>242</v>
+      </c>
+      <c r="E15" t="n">
+        <v>69</v>
+      </c>
+      <c r="F15" t="n">
         <v>173</v>
       </c>
-      <c r="E15" t="n">
-        <v>50</v>
-      </c>
-      <c r="F15" t="n">
-        <v>123</v>
-      </c>
       <c r="G15" t="n">
-        <v>28.9</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="E16" t="n">
         <v>18</v>
       </c>
       <c r="F16" t="n">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="G16" t="n">
-        <v>24</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2316</v>
+        <v>2805</v>
       </c>
       <c r="E17" t="n">
-        <v>450</v>
+        <v>515</v>
       </c>
       <c r="F17" t="n">
-        <v>1866</v>
+        <v>2290</v>
       </c>
       <c r="G17" t="n">
-        <v>19.4</v>
+        <v>18.4</v>
       </c>
     </row>
   </sheetData>
@@ -1106,22 +1106,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>77.59999999999999</v>
+        <v>78</v>
       </c>
       <c r="C2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>68</v>
+        <v>67.3</v>
       </c>
       <c r="E2" t="n">
+        <v>52</v>
+      </c>
+      <c r="F2" t="n">
         <v>50</v>
       </c>
-      <c r="F2" t="n">
-        <v>51.4</v>
-      </c>
       <c r="G2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H2" t="n">
         <v>52.5</v>
@@ -1130,31 +1130,34 @@
         <v>61</v>
       </c>
       <c r="J2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="L2" t="n">
+        <v>42.9</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N2" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="O2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P2" t="n">
-        <v>34.1</v>
+        <v>33.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="R2" t="n">
-        <v>21.9</v>
+        <v>22.1</v>
       </c>
       <c r="S2" t="n">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="T2" t="n">
         <v>28.6</v>
@@ -1163,19 +1166,22 @@
         <v>7</v>
       </c>
       <c r="V2" t="n">
-        <v>37.5</v>
+        <v>42.3</v>
       </c>
       <c r="W2" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="X2" t="n">
-        <v>26.5</v>
+        <v>28</v>
       </c>
       <c r="Y2" t="n">
-        <v>49</v>
+        <v>50</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>100</v>
       </c>
       <c r="AA2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB2" t="n">
         <v>100</v>
@@ -1187,10 +1193,10 @@
         <v>0</v>
       </c>
       <c r="AF2" t="n">
-        <v>70.09999999999999</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AG2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3">
@@ -1199,32 +1205,50 @@
           <t>Above Avg</t>
         </is>
       </c>
+      <c r="B3" t="n">
+        <v>66.7</v>
+      </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>33.3</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
+      <c r="H3" t="n">
+        <v>100</v>
+      </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
+      <c r="L3" t="n">
+        <v>19</v>
+      </c>
       <c r="M3" t="n">
+        <v>21</v>
+      </c>
+      <c r="N3" t="n">
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="P3" t="n">
+        <v>50</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R3" t="n">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="S3" t="n">
         <v>554</v>
@@ -1236,19 +1260,22 @@
         <v>5</v>
       </c>
       <c r="V3" t="n">
-        <v>38.5</v>
+        <v>31.2</v>
       </c>
       <c r="W3" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="X3" t="n">
-        <v>37.5</v>
+        <v>36.4</v>
       </c>
       <c r="Y3" t="n">
-        <v>128</v>
+        <v>132</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>66.7</v>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
@@ -1366,35 +1393,59 @@
           <t>Below Avg</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>80</v>
+      </c>
       <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>80</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="n">
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>25</v>
+      </c>
+      <c r="K5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="M5" t="n">
+        <v>11</v>
+      </c>
+      <c r="N5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" t="n">
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R5" t="n">
-        <v>15.4</v>
+        <v>18</v>
       </c>
       <c r="S5" t="n">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="T5" t="n">
         <v>25</v>
@@ -1403,16 +1454,16 @@
         <v>4</v>
       </c>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="W5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="X5" t="n">
-        <v>20</v>
+        <v>19.6</v>
       </c>
       <c r="Y5" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AA5" t="n">
         <v>0</v>
@@ -1424,10 +1475,10 @@
         <v>0</v>
       </c>
       <c r="AF5" t="n">
-        <v>100</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="AG5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -1485,7 +1536,7 @@
         <v>4</v>
       </c>
       <c r="R6" t="n">
-        <v>14.5</v>
+        <v>14.3</v>
       </c>
       <c r="S6" t="n">
         <v>519</v>
@@ -1540,100 +1591,100 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>63.5</v>
+        <v>61.1</v>
       </c>
       <c r="C7" t="n">
-        <v>496</v>
+        <v>573</v>
       </c>
       <c r="D7" t="n">
-        <v>63.3</v>
+        <v>64</v>
       </c>
       <c r="E7" t="n">
-        <v>286</v>
+        <v>336</v>
       </c>
       <c r="F7" t="n">
         <v>61.4</v>
       </c>
       <c r="G7" t="n">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="H7" t="n">
-        <v>60.9</v>
+        <v>61.5</v>
       </c>
       <c r="I7" t="n">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="J7" t="n">
-        <v>24.7</v>
+        <v>22.3</v>
       </c>
       <c r="K7" t="n">
-        <v>162</v>
+        <v>206</v>
       </c>
       <c r="L7" t="n">
-        <v>28.9</v>
+        <v>28.5</v>
       </c>
       <c r="M7" t="n">
-        <v>173</v>
+        <v>242</v>
       </c>
       <c r="N7" t="n">
-        <v>24</v>
+        <v>20.5</v>
       </c>
       <c r="O7" t="n">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="P7" t="n">
-        <v>19.4</v>
+        <v>18.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>2316</v>
+        <v>2805</v>
       </c>
       <c r="R7" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="S7" t="n">
+        <v>2424</v>
+      </c>
+      <c r="T7" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="U7" t="n">
+        <v>66</v>
+      </c>
+      <c r="V7" t="n">
+        <v>47</v>
+      </c>
+      <c r="W7" t="n">
+        <v>132</v>
+      </c>
+      <c r="X7" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>596</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>76</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>32</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="AE7" t="n">
         <v>17</v>
       </c>
-      <c r="S7" t="n">
-        <v>2411</v>
-      </c>
-      <c r="T7" t="n">
-        <v>31.7</v>
-      </c>
-      <c r="U7" t="n">
-        <v>63</v>
-      </c>
-      <c r="V7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="W7" t="n">
-        <v>118</v>
-      </c>
-      <c r="X7" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>567</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>66.09999999999999</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>62</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>26</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>16</v>
-      </c>
       <c r="AF7" t="n">
-        <v>61</v>
+        <v>60.1</v>
       </c>
       <c r="AG7" t="n">
-        <v>205</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily slate 2026-06-04 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-23.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-23.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2202</v>
+        <v>2190</v>
       </c>
       <c r="E2" t="n">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="F2" t="n">
-        <v>1826</v>
+        <v>1809</v>
       </c>
       <c r="G2" t="n">
-        <v>17.1</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="3">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E4" t="n">
         <v>47</v>
       </c>
       <c r="F4" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="G4" t="n">
-        <v>36.2</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E6" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F6" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G6" t="n">
-        <v>43.8</v>
+        <v>44.1</v>
       </c>
     </row>
     <row r="7">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>745</v>
+        <v>695</v>
       </c>
       <c r="E8" t="n">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="F8" t="n">
-        <v>503</v>
+        <v>475</v>
       </c>
       <c r="G8" t="n">
-        <v>32.5</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E9" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F9" t="n">
         <v>71</v>
       </c>
       <c r="G9" t="n">
-        <v>60.8</v>
+        <v>60.6</v>
       </c>
     </row>
     <row r="10">
@@ -1157,7 +1157,7 @@
         <v>23.4</v>
       </c>
       <c r="S2" t="n">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="T2" t="n">
         <v>44.4</v>
@@ -1172,10 +1172,10 @@
         <v>26</v>
       </c>
       <c r="X2" t="n">
-        <v>20.3</v>
+        <v>19.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="Z2" t="n">
         <v>100</v>
@@ -1248,10 +1248,10 @@
         <v>2</v>
       </c>
       <c r="R3" t="n">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="S3" t="n">
-        <v>554</v>
+        <v>547</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
@@ -1260,16 +1260,16 @@
         <v>5</v>
       </c>
       <c r="V3" t="n">
-        <v>31.2</v>
+        <v>28.6</v>
       </c>
       <c r="W3" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="X3" t="n">
-        <v>36.4</v>
+        <v>31.1</v>
       </c>
       <c r="Y3" t="n">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="Z3" t="n">
         <v>66.7</v>
@@ -1284,10 +1284,10 @@
         <v>0</v>
       </c>
       <c r="AF3" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="AG3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1345,16 +1345,16 @@
         <v>54</v>
       </c>
       <c r="R4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="S4" t="n">
+        <v>499</v>
+      </c>
+      <c r="T4" t="n">
         <v>20.8</v>
       </c>
-      <c r="S4" t="n">
-        <v>504</v>
-      </c>
-      <c r="T4" t="n">
-        <v>19.2</v>
-      </c>
       <c r="U4" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="V4" t="n">
         <v>56.2</v>
@@ -1363,10 +1363,10 @@
         <v>32</v>
       </c>
       <c r="X4" t="n">
-        <v>32</v>
+        <v>32.2</v>
       </c>
       <c r="Y4" t="n">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="Z4" t="n">
         <v>50</v>
@@ -1445,16 +1445,16 @@
         <v>2</v>
       </c>
       <c r="R5" t="n">
-        <v>18</v>
+        <v>18.6</v>
       </c>
       <c r="S5" t="n">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="T5" t="n">
-        <v>25</v>
+        <v>33.3</v>
       </c>
       <c r="U5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V5" t="n">
         <v>20</v>
@@ -1463,10 +1463,10 @@
         <v>5</v>
       </c>
       <c r="X5" t="n">
-        <v>19.6</v>
+        <v>22.5</v>
       </c>
       <c r="Y5" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AA5" t="n">
         <v>0</v>
@@ -1539,10 +1539,10 @@
         <v>4</v>
       </c>
       <c r="R6" t="n">
-        <v>14.5</v>
+        <v>14.7</v>
       </c>
       <c r="S6" t="n">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="T6" t="n">
         <v>16.7</v>
@@ -1551,16 +1551,16 @@
         <v>12</v>
       </c>
       <c r="V6" t="n">
-        <v>27.3</v>
+        <v>30</v>
       </c>
       <c r="W6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="X6" t="n">
-        <v>39.5</v>
+        <v>39.3</v>
       </c>
       <c r="Y6" t="n">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="Z6" t="n">
         <v>100</v>
@@ -1642,28 +1642,28 @@
         <v>2412</v>
       </c>
       <c r="R7" t="n">
-        <v>17.1</v>
+        <v>17.4</v>
       </c>
       <c r="S7" t="n">
-        <v>2202</v>
+        <v>2190</v>
       </c>
       <c r="T7" t="n">
-        <v>36.2</v>
+        <v>37</v>
       </c>
       <c r="U7" t="n">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="V7" t="n">
-        <v>43.8</v>
+        <v>44.1</v>
       </c>
       <c r="W7" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="X7" t="n">
-        <v>32.5</v>
+        <v>31.7</v>
       </c>
       <c r="Y7" t="n">
-        <v>745</v>
+        <v>695</v>
       </c>
       <c r="Z7" t="n">
         <v>65.2</v>
@@ -1684,10 +1684,10 @@
         <v>4</v>
       </c>
       <c r="AF7" t="n">
-        <v>60.8</v>
+        <v>60.6</v>
       </c>
       <c r="AG7" t="n">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>